<commit_message>
Mostrar la rúbrica en el dashboard del instructor, con el segundo viernes el 2 de octubre.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/recursos/instructor/Rubrica-Evaluacion-Participantes-CISA.xlsx
+++ b/recursos/instructor/Rubrica-Evaluacion-Participantes-CISA.xlsx
@@ -71,21 +71,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gladys del Socorro Mejía Chacón</t>
+          <t>Oscar Eduin Rodríguez Orellana</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gerente de Control de Calidad</t>
+          <t>Gerente de Compras, Operaciones y Logística</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>gmejia</t>
+          <t>orodriguez</t>
         </is>
       </c>
       <c r="D2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2">
         <v>24</v>
@@ -94,10 +94,10 @@
         <v>34</v>
       </c>
       <c r="G2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H2">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -106,7 +106,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>El aviso del lote que no salió</t>
+          <t>Tres proveedores, ningún ganador</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -118,17 +118,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rita Gisele Cerrato Varela</t>
+          <t>Kellyn Nazaria Escalante Andino</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gerente de Recursos Humanos</t>
+          <t>Sub-Gerente Regional</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>gcerrato</t>
+          <t>kescalante</t>
         </is>
       </c>
       <c r="D3">
@@ -138,13 +138,13 @@
         <v>24</v>
       </c>
       <c r="F3">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G3">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H3">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -153,7 +153,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>El aviso de una vacante interna</t>
+          <t>El resumen de la semana</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -165,17 +165,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kellyn Nazaria Escalante Andino</t>
+          <t>Gladys del Socorro Mejía Chacón</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sub-Gerente Regional</t>
+          <t>Gerente de Control de Calidad</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>kescalante</t>
+          <t>gmejia</t>
         </is>
       </c>
       <c r="D4">
@@ -191,7 +191,7 @@
         <v>19</v>
       </c>
       <c r="H4">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -200,7 +200,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>El resumen de la semana</t>
+          <t>El aviso del lote que no salió</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -212,64 +212,64 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hernán Danilo Zaldívar Nolasco</t>
+          <t>Marlon Mauricio Vega Rodríguez</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gerente General</t>
+          <t>Gerente de Sistemas de Información</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>dzaldivar</t>
+          <t>mvega</t>
         </is>
       </c>
       <c r="D5">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E5">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F5">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G5">
         <v>19</v>
       </c>
       <c r="H5">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Observado</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Una página para decidir</t>
+          <t>El correo se cayó 18 minutos</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Casi no asistió el segundo viernes (25 de septiembre). Baja en participación y en módulos de oficina.</t>
+          <t>Cursó las dos jornadas. Proyecto de su cargo cerrado.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Allan Fernando Baide Simon</t>
+          <t>Rita Gisele Cerrato Varela</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gerente de Ventas</t>
+          <t>Gerente de Recursos Humanos</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>abaide</t>
+          <t>gcerrato</t>
         </is>
       </c>
       <c r="D6">
@@ -285,7 +285,7 @@
         <v>19</v>
       </c>
       <c r="H6">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -294,7 +294,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>El correo después de la visita</t>
+          <t>El aviso de una vacante interna</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -306,33 +306,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oscar Eduin Rodríguez Orellana</t>
+          <t>Héctor Adolfo Dore Serrano</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gerente de Compras, Operaciones y Logística</t>
+          <t>Jefe de Desarrollo Digital y Automatización</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>orodriguez</t>
+          <t>hdore</t>
         </is>
       </c>
       <c r="D7">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G7">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H7">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -341,7 +341,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Tres proveedores, ningún ganador</t>
+          <t>Un piloto, sin conectar el sistema</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -353,21 +353,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Miguel Antonio López Briones</t>
+          <t>Allan Fernando Baide Simon</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gerente de Auditoría</t>
+          <t>Gerente de Ventas</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>mlopez</t>
+          <t>abaide</t>
         </is>
       </c>
       <c r="D8">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E8">
         <v>23</v>
@@ -376,10 +376,10 @@
         <v>32</v>
       </c>
       <c r="G8">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H8">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -388,7 +388,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Qué se arriesga si usan un chat</t>
+          <t>El correo después de la visita</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -400,17 +400,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gerardo Enrique Paredes Lontero</t>
+          <t>Miguel Antonio López Briones</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gerente de Producción</t>
+          <t>Gerente de Auditoría</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>gparedes</t>
+          <t>mlopez</t>
         </is>
       </c>
       <c r="D9">
@@ -423,10 +423,10 @@
         <v>32</v>
       </c>
       <c r="G9">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H9">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -435,7 +435,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>El papel del relevo de turno</t>
+          <t>Qué se arriesga si usan un chat</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -447,33 +447,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Marlon Mauricio Vega Rodríguez</t>
+          <t>Gerardo Enrique Paredes Lontero</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gerente de Sistemas de Información</t>
+          <t>Gerente de Producción</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>mvega</t>
+          <t>gparedes</t>
         </is>
       </c>
       <c r="D10">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E10">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F10">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G10">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H10">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -482,7 +482,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>El correo se cayó 18 minutos</t>
+          <t>El papel del relevo de turno</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -494,47 +494,47 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Héctor Adolfo Dore Serrano</t>
+          <t>Hernán Danilo Zaldívar Nolasco</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Jefe de Desarrollo Digital y Automatización</t>
+          <t>Gerente General</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>hdore</t>
+          <t>dzaldivar</t>
         </is>
       </c>
       <c r="D11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F11">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G11">
         <v>19</v>
       </c>
       <c r="H11">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Un piloto, sin conectar el sistema</t>
+          <t>Una página para decidir</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Cursó las dos jornadas. Proyecto de su cargo cerrado.</t>
+          <t>Casi no asistió el segundo viernes (2 de octubre de 2026). Baja en participación y en módulos de oficina.</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Asistencia a los dos viernes. Prácticas y comparación de los dos chats.</t>
+          <t>Asistencia a los dos viernes. Prácticas y los dos chats.</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hernán Danilo Zaldívar Nolasco: 75. Casi no entró el 2.º viernes.</t>
+          <t>Danilo Zaldívar: 75. Casi no entró el viernes 2 de octubre.</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11 y 25 de septiembre de 2026. San Pedro Sula. Magnatic para CISA.</t>
+          <t>Viernes 11 de septiembre y viernes 2 de octubre de 2026. San Pedro Sula. Magnatic para CISA.</t>
         </is>
       </c>
     </row>

</xml_diff>